<commit_message>
memoria: auto-refresh resumo + dashboard (18:15 task)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/memoria/memoria-resumo.xlsx
+++ b/memoria/memoria-resumo.xlsx
@@ -3808,10 +3808,10 @@
         <v>1120</v>
       </c>
       <c r="I7" t="n">
-        <v>975.5599999999999</v>
+        <v>940.4400000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>165.44</v>
+        <v>164.51</v>
       </c>
     </row>
     <row r="8">
@@ -3842,10 +3842,10 @@
         <v>728</v>
       </c>
       <c r="I8" t="n">
-        <v>2229000</v>
+        <v>1828000</v>
       </c>
       <c r="J8" t="n">
-        <v>595061.38</v>
+        <v>618346.73</v>
       </c>
     </row>
     <row r="9">
@@ -3876,10 +3876,10 @@
         <v>5969</v>
       </c>
       <c r="I9" t="n">
-        <v>290500</v>
+        <v>257500</v>
       </c>
       <c r="J9" t="n">
-        <v>67535.34</v>
+        <v>69993.14999999999</v>
       </c>
     </row>
     <row r="10">
@@ -3910,10 +3910,10 @@
         <v>540</v>
       </c>
       <c r="I10" t="n">
-        <v>76260</v>
+        <v>67100</v>
       </c>
       <c r="J10" t="n">
-        <v>12123.54</v>
+        <v>12620.8</v>
       </c>
     </row>
     <row r="11">
@@ -3944,10 +3944,10 @@
         <v>145</v>
       </c>
       <c r="I11" t="n">
-        <v>1745</v>
+        <v>1755</v>
       </c>
       <c r="J11" t="n">
-        <v>214.99</v>
+        <v>222.72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>